<commit_message>
Implement supplement recommendation flow
</commit_message>
<xml_diff>
--- a/AI 知识库.xlsx
+++ b/AI 知识库.xlsx
@@ -11180,12 +11180,12 @@
           <t>生产中</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026年5月底</t>
-        </is>
-      </c>
-      <c r="E2"/>
+      <c r="D2"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>物流清关情况确认后</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>通用话术</t>
@@ -11201,7 +11201,7 @@
         </is>
       </c>
       <c r="J2" s="2">
-        <v>46150.52780092593</v>
+        <v>46175.76115740741</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>

</xml_diff>